<commit_message>
Select 2017 for TX-123BT, fix scenario name in NREL-118
</commit_message>
<xml_diff>
--- a/data/TX-123BT/Global_Scenarios.xlsx
+++ b/data/TX-123BT/Global_Scenarios.xlsx
@@ -714,7 +714,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B9" s="11" t="n">
         <v/>
       </c>
@@ -733,7 +737,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B10" s="11" t="n">
         <v/>
       </c>
@@ -752,7 +760,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B11" s="11" t="n">
         <v/>
       </c>
@@ -771,7 +783,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B12" s="11" t="n">
         <v/>
       </c>

</xml_diff>